<commit_message>
Update 1_formulas | comparision operators & cell referencing
</commit_message>
<xml_diff>
--- a/2_Formulas_Functions/1_Formulas.xlsx
+++ b/2_Formulas_Functions/1_Formulas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7456b23f02075ab8/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7456b23f02075ab8/Documents/Excel LUKE/2_Formulas_Functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{12E7163F-7AE5-448A-922E-9D1EC6C65849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{12E7163F-7AE5-448A-922E-9D1EC6C65849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B128F5D-77FB-4C4E-BFDC-7636917F69B1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7154411A-786C-4E27-A87D-140983770EDC}"/>
   </bookViews>
@@ -685,13 +685,17 @@
     <col min="3" max="3" width="10.44140625" style="1" customWidth="1"/>
     <col min="4" max="4" width="12.21875" style="1" customWidth="1"/>
     <col min="5" max="5" width="11.5546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10" style="1" customWidth="1"/>
-    <col min="7" max="8" width="9" style="1"/>
-    <col min="9" max="9" width="18.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.21875" style="1" customWidth="1"/>
-    <col min="11" max="13" width="9" style="1"/>
-    <col min="14" max="14" width="11.21875" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="9" style="1"/>
+    <col min="6" max="6" width="12.88671875" style="1" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.21875" style="1" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="18.21875" style="1" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="33.33203125" style="1" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="22.6640625" style="1" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -768,6 +772,30 @@
         <f>D3*H3+D3</f>
         <v>130000</v>
       </c>
+      <c r="J3" s="1" t="b">
+        <f>G3=I3</f>
+        <v>1</v>
+      </c>
+      <c r="K3" s="1" t="b">
+        <f>E3&gt;D3</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="1" t="b">
+        <f>$C$15&lt;=C3</f>
+        <v>1</v>
+      </c>
+      <c r="M3" s="1" t="b">
+        <f>G3&gt;=$C$16</f>
+        <v>1</v>
+      </c>
+      <c r="N3" s="1">
+        <f>L3*M3</f>
+        <v>1</v>
+      </c>
+      <c r="O3" s="1" t="b">
+        <f>N3=1</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
@@ -783,7 +811,7 @@
         <v>12000</v>
       </c>
       <c r="F4" s="1">
-        <f t="shared" ref="F4:F13" si="0">C4</f>
+        <f t="shared" ref="F4:F12" si="0">C4</f>
         <v>4</v>
       </c>
       <c r="G4" s="1">
@@ -797,6 +825,30 @@
       <c r="I4" s="1">
         <f t="shared" ref="I4:I12" si="3">D4*H4+D4</f>
         <v>147000</v>
+      </c>
+      <c r="J4" s="1" t="b">
+        <f t="shared" ref="J4:J12" si="4">G4=I4</f>
+        <v>1</v>
+      </c>
+      <c r="K4" s="1" t="b">
+        <f t="shared" ref="K4:K12" si="5">E4&gt;D4</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="1" t="b">
+        <f t="shared" ref="L4:L12" si="6">$C$15&lt;=C4</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="1" t="b">
+        <f t="shared" ref="M4:M12" si="7">G4&gt;=$C$16</f>
+        <v>1</v>
+      </c>
+      <c r="N4" s="1">
+        <f t="shared" ref="N4:N12" si="8">L4*M4</f>
+        <v>0</v>
+      </c>
+      <c r="O4" s="1" t="b">
+        <f t="shared" ref="O4:O12" si="9">N4=1</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
@@ -828,6 +880,30 @@
         <f t="shared" si="3"/>
         <v>80000</v>
       </c>
+      <c r="J5" s="1" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K5" s="1" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L5" s="1" t="b">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="M5" s="1" t="b">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="N5" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="1" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
@@ -858,6 +934,30 @@
         <f t="shared" si="3"/>
         <v>118000</v>
       </c>
+      <c r="J6" s="1" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K6" s="1" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L6" s="1" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="M6" s="1" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="N6" s="1">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="O6" s="1" t="b">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
@@ -888,6 +988,30 @@
         <f t="shared" si="3"/>
         <v>136000</v>
       </c>
+      <c r="J7" s="1" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K7" s="1" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L7" s="1" t="b">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="M7" s="1" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="N7" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="O7" s="1" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
@@ -918,6 +1042,30 @@
         <f t="shared" si="3"/>
         <v>97000</v>
       </c>
+      <c r="J8" s="1" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K8" s="1" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L8" s="1" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="M8" s="1" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="N8" s="1">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="O8" s="1" t="b">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
@@ -948,6 +1096,30 @@
         <f t="shared" si="3"/>
         <v>165000</v>
       </c>
+      <c r="J9" s="1" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K9" s="1" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L9" s="1" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="M9" s="1" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="N9" s="1">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="O9" s="1" t="b">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
@@ -978,6 +1150,30 @@
         <f t="shared" si="3"/>
         <v>143000</v>
       </c>
+      <c r="J10" s="1" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K10" s="1" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L10" s="1" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="M10" s="1" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="N10" s="1">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="O10" s="1" t="b">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
@@ -1008,6 +1204,30 @@
         <f t="shared" si="3"/>
         <v>154000</v>
       </c>
+      <c r="J11" s="1" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K11" s="1" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L11" s="1" t="b">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="M11" s="1" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="N11" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="O11" s="1" t="b">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="10" t="s">
@@ -1038,6 +1258,30 @@
         <f t="shared" si="3"/>
         <v>124000</v>
       </c>
+      <c r="J12" s="1" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K12" s="1" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="L12" s="1" t="b">
+        <f t="shared" si="6"/>
+        <v>1</v>
+      </c>
+      <c r="M12" s="1" t="b">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
+      <c r="N12" s="1">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="O12" s="1" t="b">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="13" t="s">
@@ -1048,13 +1292,17 @@
       <c r="B15" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="15"/>
+      <c r="C15" s="15">
+        <v>5</v>
+      </c>
     </row>
     <row r="16" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="17"/>
+      <c r="C16" s="17">
+        <v>90000</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>